<commit_message>
Add true-everything experiment results and updated documentation
- true_everything_50M: 57% Story QA (all mods + QA + sparsity + copy gate)
- true_everything_no_qa_50M: 15% Story QA (same but NO QA data)
- Updated FINAL_EXP.xlsx with 2 new rows, striped by token training tier
- Updated PROCESS.md and RESULTS.md for true-everything branch

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiment_tracker.xlsx
+++ b/experiment_tracker.xlsx
@@ -1,16 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Experiments" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dataset_Overview" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Examples_everything_optimized_5" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Examples_everything_50M_rerun" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset_Overview" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_everything_optimized_5" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_everything_50M_rerun" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_true_everything_50M" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_true_everything_no_qa_" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -661,6 +663,110 @@
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>2026-02-27 03:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>true_everything_50M</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>True everything (all mods + QA data + sparsity + copy gate)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Does combining ALL modifications improve Story QA beyond data augmentation alone?</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>78,913,436</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>17.15%</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>57.0%</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>checkpoints/true_everything_copy_gate_50M.pt</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27 06:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>true_everything_no_qa_50M</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>True everything (all mods + sparsity + copy gate, NO QA data)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Isolate architectural mods: do sparsity + copy gate help without QA data?</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>78,896,305</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>17.17%</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>15.0%</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>checkpoints/true_everything_no_qa_copy_gate_50M.pt</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27 06:24</t>
         </is>
       </c>
     </row>
@@ -2287,4 +2393,1344 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Doc ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Story (truncated)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Words</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t># Questions</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Test Question</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Gold Answer</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Model Answer</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Match?</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Story Loss</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Story PPL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Avg Confidence</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Top-5 for 1st Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_067101</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>The cat sat on the mat. It was time for a nap. He curled up in a ball. What a good time!</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Where did the cat sit?</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>The cat sat on the mat.</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>The cat sit on the mat.</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>4.4641</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>86.84</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>58.67%</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The(82%) |  When(2%) |  A(1%) |  What(1%) |  According(1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_084814</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>A little microtus lived in a tree. He resolved to be brave. He learned to fly. He flew in the sky!</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Where did the little microtus live?</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>He lived in a tree.</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>The little microtus live in a tree.</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>4.7466</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>115.19</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>68.25%</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The(80%) |  When(2%) |  He(2%) |  A(1%) |  No(1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_021609</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Timmy had two toy cars. He was a member of the car club. It was hard to pick a favorite car. He felt confused. The blue car had a pull cord.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>How many toy cars did Timmy have?</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Timmy had two toy cars.</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>The car was a car club with the car club.</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>4.1530</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>63.63</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>34.25%</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Tim(36%) |  The(24%) |  According(7%) |  Three(1%) |  A(1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_006447</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Tim loved candy. Candy was his vice. He ate candy every day. One day, Tim dreamed he was in Germany. Everything was made of candy! The houses were as big as mountains. He saw a real candy dragon. The dragon was nice. It gave Tim a lollipop. Tim woke up. He wanted more candy!</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>What did Tim love?</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Tim loved candy.</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Tim did not like candy. The dragon did not like candy.</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>4.7105</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>111.10</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>35.46%</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Tim(92%) |  The(4%) |  When(0%) |  According(0%) |  He(0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_096600</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>The cat saw many things. There were toys on the floor. There was a bird outside. The cat noted the bird. "I want to play with the bird," she thought. But the bird was in a tree. The tree was too tall. The cat could not climb it. She went back inside. She played with a toy instead. It was a fun day.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>What did the cat see?</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>The cat saw toys and a bird.</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>The cat saw many things.</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>3.4499</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>31.50</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>67.95%</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The(97%) |  According(1%) |  When(0%) |  After(0%) |  A(0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_051870</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>The teddy bear was old. His fur was worn. He loved to play. He lived in a toy box. The toy box was in a messy state. One day, a girl picked him up. She wanted to convey a message. She put him on a chair. She made him hold a note. The note said, "I love you." The teddy bear helped to convey her feeli</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>What kind of bear was it?</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>It was a teddy bear.</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>A girl picked me up.</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>3.5553</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>35.00</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>34.81%</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The(68%) |  A(13%) |  According(5%) |  When(3%) |  It(1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_062893</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>The snake was long. It was also sinuous. It moved like a ribbon. The snake lived in a big tree. It liked to sleep in the sun. One day, a bird landed on the tree. The bird saw the snake. It was as green as the leaves. The snake looked at the bird. The bird chirped. The snake moved slowly. It made a s</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>What animal is in the story?</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>A snake is in the story.</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>The snake was long. It is called a snake. It was a human. The snake was long.</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>3.4329</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>30.97</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>42.88%</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The(84%) |  According(4%) |  A(2%) |  In(2%) |  When(1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_093253</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The little frog was green. He lived by a big rock. The rock was grey. One day, the frog wanted to play. He looked left. He looked right. He saw a fly! The fly was buzzing between two big leaves. The frog jumped high. He wanted to catch the fly. But the fly flew away! The frog was sad. He sat on the </t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>What color was the little frog?</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>The frog was green.</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>The little frog was green. They had a green cannon.</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>3.7484</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>42.45</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>48.46%</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The(96%) |  According(1%) |  When(0%) |  A(0%) |  He(0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_003445</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>The big bus had a flat tire. Oh no! That was not good. The bus could not go. The driver looked sad. He needed to fix it. This was part of his job. “I can help!” said Tim. Tim was only one small boy. But he was strong. “How?” asked the driver. “I can hold the light!” said Tim. The driver smiled. He g</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>126</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>What happened to the big bus?</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>The bus had a flat tire.</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Tim was only one small boy. He was happy to help. He had a flat tire. Tim's driver was happy to help.</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>3.5106</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>33.47</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>51.95%</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Tim(52%) |  The(40%) |  According(2%) |  When(1%) |  No(1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_011051</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The pig liked to play tricks. He would act silly. He did it in a funny manner. He would run and jump. He would make silly faces. He did it over and over. This is called repetition. One day, the farmer saw the pig. The farmer did not like the pig's tricks. The farmer yelled, "Stop that!" The pig did </t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>125</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>What did the pig like to do?</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>The pig liked to play tricks.</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>The pig liked to play tricks because he was fast. He did this by getting the farmer to throw the pig. He did it over.</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>3.4897</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>32.78</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>40.32%</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The(97%) |  According(1%) |  When(0%) |  He(0%) |  the(0%)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Doc ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Story (truncated)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Words</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t># Questions</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Test Question</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Gold Answer</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Model Answer</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Match?</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Story Loss</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Story PPL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Avg Confidence</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Top-5 for 1st Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_067101</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>The cat sat on the mat. It was time for a nap. He curled up in a ball. What a good time!</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Where did the cat sit?</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>The cat sat on the mat.</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>What type of cat sitting?</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>4.4226</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>83.32</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>41.01%</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> What(13%) |  When(9%) |  The(9%) |  How(7%) |  Where(5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_084814</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>A little microtus lived in a tree. He resolved to be brave. He learned to fly. He flew in the sky!</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Where did the little microtus live?</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>He lived in a tree.</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>How did the little microtus survive in the sky?</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>4.5903</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>98.52</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>49.67%</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> What(14%) |  How(11%) |  When(7%) |  The(7%) |  Where(5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_021609</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Timmy had two toy cars. He was a member of the car club. It was hard to pick a favorite car. He felt confused. The blue car had a pull cord.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>How many toy cars did Timmy have?</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Timmy had two toy cars.</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>The trick is to pick a favorite car for the car. The car is in the lower side.</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>4.0666</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>58.36</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>23.24%</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> What(10%) |  The(9%) |  Tim(8%) |  How(6%) |  When(5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_006447</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Tim loved candy. Candy was his vice. He ate candy every day. One day, Tim dreamed he was in Germany. Everything was made of candy! The houses were as big as mountains. He saw a real candy dragon. The dragon was nice. It gave Tim a lollipop. Tim woke up. He wanted more candy!</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>What did Tim love?</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Tim loved candy.</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Tim could not eat candy! He knew she didn’t eat candy on his own. Tim wanted to eat candy! Tim didn’t eat candy because he ate candy. Tim didn’t eat candy because Tim’s up-to-date. Tim took a look at</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>4.7631</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>117.11</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>42.71%</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Tim(70%) |  The(2%) |  He(2%) |  What(2%) |  When(1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_096600</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>The cat saw many things. There were toys on the floor. There was a bird outside. The cat noted the bird. "I want to play with the bird," she thought. But the bird was in a tree. The tree was too tall. The cat could not climb it. She went back inside. She played with a toy instead. It was a fun day.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>What did the cat see?</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>The cat saw toys and a bird.</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Why did the cat go back inside?</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>3.4703</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>32.15</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>42.06%</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The(19%) |  What(13%) |  "(5%) |  How(5%) |  When(4%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_051870</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>The teddy bear was old. His fur was worn. He loved to play. He lived in a toy box. The toy box was in a messy state. One day, a girl picked him up. She wanted to convey a message. She put him on a chair. She made him hold a note. The note said, "I love you." The teddy bear helped to convey her feeli</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>What kind of bear was it?</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>It was a teddy bear.</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>If you have a teddy bears, you are not sure how many bear we have. It is not known what it is.</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>3.5193</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>33.76</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>21.43%</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> What(22%) |  The(8%) |  How(5%) |  When(4%) |  Why(4%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_062893</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>The snake was long. It was also sinuous. It moved like a ribbon. The snake lived in a big tree. It liked to sleep in the sun. One day, a bird landed on the tree. The bird saw the snake. It was as green as the leaves. The snake looked at the bird. The bird chirped. The snake moved slowly. It made a s</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>What animal is in the story?</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>A snake is in the story.</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>How animal is in the story?</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>3.4374</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>31.11</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>59.44%</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> What(17%) |  The(15%) |  How(6%) |  When(4%) |  Why(4%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_093253</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The little frog was green. He lived by a big rock. The rock was grey. One day, the frog wanted to play. He looked left. He looked right. He saw a fly! The fly was buzzing between two big leaves. The frog jumped high. He wanted to catch the fly. But the fly flew away! The frog was sad. He sat on the </t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>What color was the little frog?</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>The frog was green.</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>What color was the no big frog?</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>3.5696</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>35.50</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>47.41%</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> What(23%) |  The(10%) |  How(9%) |  Why(5%) |  Which(4%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_003445</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>The big bus had a flat tire. Oh no! That was not good. The bus could not go. The driver looked sad. He needed to fix it. This was part of his job. “I can help!” said Tim. Tim was only one small boy. But he was strong. “How?” asked the driver. “I can hold the light!” said Tim. The driver smiled. He g</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>126</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>What happened to the big bus?</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>The bus had a flat tire.</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Tim was full of things. Tim’s four things. Tim was a small man. He made an average of five things. Tim was a small man. Tim was big. Tim was a big man. He had a very bad man. Tim did. Tim was a big man. Tim</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>3.4529</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>31.59</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>35.04%</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Tim(51%) |  The(10%) |  What(4%) |  When(3%) |  �(2%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>story_qa_011051</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The pig liked to play tricks. He would act silly. He did it in a funny manner. He would run and jump. He would make silly faces. He did it over and over. This is called repetition. One day, the farmer saw the pig. The farmer did not like the pig's tricks. The farmer yelled, "Stop that!" The pig did </t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>125</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>What did the pig like to do?</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>The pig liked to play tricks.</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>What made the pig to do?</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>3.3317</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>27.99</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>43.85%</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> What(21%) |  The(14%) |  When(10%) |  Which(4%) |  How(4%)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>